<commit_message>
test: add TC-01 to TC-26 test cases with CSV and Excel sheets
</commit_message>
<xml_diff>
--- a/02-test-cases/Financial_Reconciliation_Cases.xlsx
+++ b/02-test-cases/Financial_Reconciliation_Cases.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -263,10 +263,55 @@
     <t>Urgent Packaging Tape, Logistics &amp; Counter Consumables</t>
   </si>
   <si>
+    <t>TC-24</t>
+  </si>
+  <si>
+    <t>Financial Reports (P&amp;L)</t>
+  </si>
+  <si>
+    <t>Operating Expenses Dynamic Reconciliation vs Paid Vouchers</t>
+  </si>
+  <si>
+    <t>/admin/reports/profit-loss</t>
+  </si>
+  <si>
+    <t>FAIL (BUG-114)</t>
+  </si>
+  <si>
+    <t>TC-25</t>
+  </si>
+  <si>
+    <t>Financial Reports (AP)</t>
+  </si>
+  <si>
+    <t>Supplier Payments Cumulative Invariant Period &lt;= All-Time</t>
+  </si>
+  <si>
+    <t>/admin/reports/supplier-payments</t>
+  </si>
+  <si>
+    <t>FAIL (BUG-109)</t>
+  </si>
+  <si>
+    <t>TC-26</t>
+  </si>
+  <si>
+    <t>Financial Reports (Sales)</t>
+  </si>
+  <si>
+    <t>Sales Report Return Deduction &amp; Netting Invariance</t>
+  </si>
+  <si>
+    <t>/admin/reports/sales</t>
+  </si>
+  <si>
+    <t>FAIL (BUG-118)</t>
+  </si>
+  <si>
     <t>TOTAL AUDITED</t>
   </si>
   <si>
-    <t>Zero-Variance Parity Invariant</t>
+    <t>Zero-Variance Baseline Invariant</t>
   </si>
   <si>
     <t>0.00 VARIANCE</t>
@@ -370,7 +415,7 @@
 <file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Financial Reconciliation (23 TC)" sheetId="1" r:id="rId1"/>
+    <sheet name="Financial Reconciliation (26 TC)" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -379,15 +424,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1158,32 +1203,128 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" t="s" s="1">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="B25" s="1"/>
-      <c r="C25" t="s" s="1">
+      <c r="B25" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1">
+      <c r="C25" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="D25" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="E25" s="3">
+        <v>0</v>
+      </c>
+      <c r="F25" s="3">
+        <v>6300</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3">
+        <v>0</v>
+      </c>
+      <c r="I25" s="3">
+        <v>24300</v>
+      </c>
+      <c r="J25" t="s" s="5">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="B26" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="C26" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="D26" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="E26" s="3">
+        <v>0</v>
+      </c>
+      <c r="F26" s="3">
+        <v>193100</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3">
+        <v>0</v>
+      </c>
+      <c r="I26" s="3">
+        <v>0</v>
+      </c>
+      <c r="J26" t="s" s="5">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="B27" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="C27" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="D27" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="E27" s="3">
+        <v>151000</v>
+      </c>
+      <c r="F27" s="3">
+        <v>25500</v>
+      </c>
+      <c r="G27" s="3">
+        <v>0</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>125500</v>
+      </c>
+      <c r="J27" t="s" s="5">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" t="s" s="1">
+        <v>102</v>
+      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" t="s" s="1">
+        <v>103</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1">
         <v>158500</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F28" s="1">
         <v>156000</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G28" s="1">
         <v>1500</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H28" s="1">
         <v>1000</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I28" s="1">
         <v>2500</v>
       </c>
-      <c r="J25" t="s" s="1">
-        <v>89</v>
+      <c r="J28" t="s" s="1">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>